<commit_message>
Versión 0.6.5 Error en integraciónes y multifilltros.
</commit_message>
<xml_diff>
--- a/outputs/Maestro.xlsx
+++ b/outputs/Maestro.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Antivirus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,76 +425,180 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Nombre</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Rol</t>
+          <t>SERIE</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>usuario Activo</t>
+          <t>RESPONSABLE</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>CEDULA</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>USUARIO DE RED</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre PC en Ab</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>VAL_NOM_INV_MAN_VS_AB</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>USER_ABSOLUTE</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>LOGUEO VS USER RED</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>FECHA DE ULTIMA CONEXIÓN ABS</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ANIVIRUS</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ANT_VS_USER</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ANALISIS VALIDACIONES</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>ESTADOCC_GEN_USUARIO</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>VAL_NOMUSUARIO_REDARANDA</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>VAL_ALIAS_REDARANDA</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>ESTADO ALIAS EN DA</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>NOMBRE EQUIPO ABSOLUTE</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>ANTIVIRUS</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>nombre 1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>guardarandita</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>activo</t>
-        </is>
-      </c>
+          <t>Produccion</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nombre 2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>guarda</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>inactivo</t>
-        </is>
-      </c>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nombre 3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>presidencia</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>inactivo</t>
-        </is>
-      </c>
+          <t>Custodia</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>